<commit_message>
added a temp drop for the outlet water on condensers
</commit_message>
<xml_diff>
--- a/main_balance.xlsx
+++ b/main_balance.xlsx
@@ -3625,7 +3625,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>8 condensers | return = 9,679,853 lb/hr @ 134.4 °F | makeup = 936,661 lb/hr</t>
+          <t>8 condensers | return = 10,755,536 lb/hr @ 129.3 °F | makeup = 1,042,797 lb/hr</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -3720,13 +3720,13 @@
         </is>
       </c>
       <c r="C40" s="25" t="n">
-        <v>9218000.302959621</v>
+        <v>10293683.5372025</v>
       </c>
       <c r="D40" s="25" t="n">
-        <v>18510.04076899522</v>
+        <v>20670.04726345883</v>
       </c>
       <c r="E40" s="27" t="n">
-        <v>83.47581720581169</v>
+        <v>83.48043221691825</v>
       </c>
     </row>
     <row r="41">
@@ -3739,13 +3739,13 @@
         </is>
       </c>
       <c r="C41" s="22" t="n">
-        <v>9679852.737523161</v>
+        <v>10755535.97176604</v>
       </c>
       <c r="D41" s="22" t="n">
-        <v>19437.45529623124</v>
+        <v>21597.46179069485</v>
       </c>
       <c r="E41" s="24" t="n">
-        <v>134.4186035896276</v>
+        <v>129.3281277734005</v>
       </c>
     </row>
     <row r="42">
@@ -3758,10 +3758,10 @@
         </is>
       </c>
       <c r="C42" s="25" t="n">
-        <v>430528.3247174657</v>
+        <v>429095.4955450651</v>
       </c>
       <c r="D42" s="25" t="n">
-        <v>864.5147082680032</v>
+        <v>861.6375412551508</v>
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
@@ -3775,13 +3775,13 @@
         </is>
       </c>
       <c r="C43" s="22" t="n">
-        <v>967985.2737523161</v>
+        <v>1075553.597176604</v>
       </c>
       <c r="D43" s="22" t="n">
-        <v>1943.745529623125</v>
+        <v>2159.746179069485</v>
       </c>
       <c r="E43" s="24" t="n">
-        <v>134.4186035896276</v>
+        <v>129.3281277734005</v>
       </c>
     </row>
     <row r="44">
@@ -3794,10 +3794,10 @@
         </is>
       </c>
       <c r="C44" s="25" t="n">
-        <v>936661.1639062427</v>
+        <v>1042796.658158127</v>
       </c>
       <c r="D44" s="25" t="n">
-        <v>1880.845710655106</v>
+        <v>2093.969193088609</v>
       </c>
       <c r="E44" s="27" t="n">
         <v>70</v>
@@ -3881,19 +3881,19 @@
         <v>1011.249247318053</v>
       </c>
       <c r="E48" s="33" t="n">
-        <v>86.42507599061878</v>
+        <v>86.85239436054502</v>
       </c>
       <c r="F48" s="22" t="n">
-        <v>1443302.772987539</v>
+        <v>1582718.339021135</v>
       </c>
       <c r="G48" s="22" t="n">
-        <v>2884.298107489086</v>
+        <v>3162.906352959903</v>
       </c>
       <c r="H48" s="24" t="n">
-        <v>143.355890609762</v>
+        <v>138.355890609762</v>
       </c>
       <c r="I48" s="22" t="n">
-        <v>1528766.446972788</v>
+        <v>1668182.013006385</v>
       </c>
     </row>
     <row r="49">
@@ -3912,19 +3912,19 @@
         <v>1011.249247318053</v>
       </c>
       <c r="E49" s="34" t="n">
-        <v>49.42522625424751</v>
+        <v>49.66960332738417</v>
       </c>
       <c r="F49" s="25" t="n">
-        <v>825403.5682425691</v>
+        <v>905133.2741825728</v>
       </c>
       <c r="G49" s="25" t="n">
-        <v>1649.48754644798</v>
+        <v>1808.819492770929</v>
       </c>
       <c r="H49" s="27" t="n">
-        <v>143.355890609762</v>
+        <v>138.355890609762</v>
       </c>
       <c r="I49" s="25" t="n">
-        <v>874278.9828699013</v>
+        <v>954008.6888099051</v>
       </c>
     </row>
     <row r="50">
@@ -3943,19 +3943,19 @@
         <v>1017.228576695272</v>
       </c>
       <c r="E50" s="33" t="n">
-        <v>40.07602197251683</v>
+        <v>40.27300828852613</v>
       </c>
       <c r="F50" s="22" t="n">
-        <v>807869.3796755079</v>
+        <v>902932.8201014427</v>
       </c>
       <c r="G50" s="22" t="n">
-        <v>1614.447201589744</v>
+        <v>1804.422102520869</v>
       </c>
       <c r="H50" s="24" t="n">
-        <v>133.0828737186033</v>
+        <v>128.0828737186033</v>
       </c>
       <c r="I50" s="22" t="n">
-        <v>847266.6428773677</v>
+        <v>942330.0833033025</v>
       </c>
     </row>
     <row r="51">
@@ -3974,19 +3974,19 @@
         <v>1019.563890979194</v>
       </c>
       <c r="E51" s="34" t="n">
-        <v>7.962371261173675</v>
+        <v>8.001419188094305</v>
       </c>
       <c r="F51" s="25" t="n">
-        <v>174675.9968543457</v>
+        <v>197181.06176574</v>
       </c>
       <c r="G51" s="25" t="n">
-        <v>349.0727355202752</v>
+        <v>394.0468860226619</v>
       </c>
       <c r="H51" s="27" t="n">
-        <v>129.059477265374</v>
+        <v>124.059477265374</v>
       </c>
       <c r="I51" s="25" t="n">
-        <v>182485.5822384717</v>
+        <v>204990.6471498659</v>
       </c>
     </row>
     <row r="52">
@@ -4005,19 +4005,19 @@
         <v>1024.996584701115</v>
       </c>
       <c r="E52" s="33" t="n">
-        <v>24.87623682952647</v>
+        <v>24.99758473058694</v>
       </c>
       <c r="F52" s="22" t="n">
-        <v>687048.6518103256</v>
+        <v>801133.4463019063</v>
       </c>
       <c r="G52" s="22" t="n">
-        <v>1372.998904497053</v>
+        <v>1600.986103720836</v>
       </c>
       <c r="H52" s="24" t="n">
-        <v>119.6832047961655</v>
+        <v>114.6832047961655</v>
       </c>
       <c r="I52" s="22" t="n">
-        <v>711318.2320224199</v>
+        <v>825403.0265140006</v>
       </c>
     </row>
     <row r="53">
@@ -4036,19 +4036,19 @@
         <v>1017.385031485097</v>
       </c>
       <c r="E53" s="34" t="n">
-        <v>143.4724126263661</v>
+        <v>144.1775164375404</v>
       </c>
       <c r="F53" s="25" t="n">
-        <v>2907968.574443268</v>
+        <v>3252144.376847562</v>
       </c>
       <c r="G53" s="25" t="n">
-        <v>5811.288118391823</v>
+        <v>6499.089482109436</v>
       </c>
       <c r="H53" s="27" t="n">
-        <v>132.8134936467732</v>
+        <v>127.8134936467732</v>
       </c>
       <c r="I53" s="25" t="n">
-        <v>3048989.336678129</v>
+        <v>3393165.139082422</v>
       </c>
     </row>
     <row r="54">
@@ -4067,19 +4067,19 @@
         <v>1017.385031485097</v>
       </c>
       <c r="E54" s="33" t="n">
-        <v>68.12857194768181</v>
+        <v>68.46339391694271</v>
       </c>
       <c r="F54" s="22" t="n">
-        <v>1380863.000899644</v>
+        <v>1544296.552252937</v>
       </c>
       <c r="G54" s="22" t="n">
-        <v>2759.518387089616</v>
+        <v>3086.12420514176</v>
       </c>
       <c r="H54" s="24" t="n">
-        <v>132.8134936467732</v>
+        <v>127.8134936467732</v>
       </c>
       <c r="I54" s="22" t="n">
-        <v>1447827.394751825</v>
+        <v>1611260.946105118</v>
       </c>
     </row>
     <row r="55">
@@ -4098,19 +4098,19 @@
         <v>1017.385031485097</v>
       </c>
       <c r="E55" s="34" t="n">
-        <v>48.88714244488114</v>
+        <v>49.12740125021033</v>
       </c>
       <c r="F55" s="25" t="n">
-        <v>990868.3580464221</v>
+        <v>1108143.666729201</v>
       </c>
       <c r="G55" s="25" t="n">
-        <v>1980.15259401763</v>
+        <v>2214.515720881696</v>
       </c>
       <c r="H55" s="27" t="n">
-        <v>132.8134936467732</v>
+        <v>127.8134936467732</v>
       </c>
       <c r="I55" s="25" t="n">
-        <v>1038920.119112259</v>
+        <v>1156195.427795038</v>
       </c>
     </row>
     <row r="56">
@@ -4125,17 +4125,17 @@
       <c r="C56" s="16" t="inlineStr"/>
       <c r="D56" s="16" t="inlineStr"/>
       <c r="E56" s="35" t="n">
-        <v>469.2530593270124</v>
+        <v>471.56232149983</v>
       </c>
       <c r="F56" s="28" t="n">
-        <v>9218000.302959621</v>
+        <v>10293683.5372025</v>
       </c>
       <c r="G56" s="28" t="n">
-        <v>18421.26359504321</v>
+        <v>20570.91034612809</v>
       </c>
       <c r="H56" s="16" t="inlineStr"/>
       <c r="I56" s="28" t="n">
-        <v>9679852.737523161</v>
+        <v>10755535.97176604</v>
       </c>
     </row>
     <row r="57">
@@ -4145,7 +4145,7 @@
         </is>
       </c>
       <c r="B57" s="30" t="n">
-        <v>83.47581720581169</v>
+        <v>83.48043221691825</v>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="B60" s="7" t="n">
-        <v>9218000.302959621</v>
+        <v>10293683.5372025</v>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
@@ -4205,7 +4205,7 @@
         </is>
       </c>
       <c r="B62" s="7" t="n">
-        <v>9679852.737523161</v>
+        <v>10755535.97176604</v>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
@@ -4220,7 +4220,7 @@
         </is>
       </c>
       <c r="B63" s="7" t="n">
-        <v>19437.45529623124</v>
+        <v>21597.46179069485</v>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
@@ -4235,7 +4235,7 @@
         </is>
       </c>
       <c r="B64" s="30" t="n">
-        <v>134.4186035896276</v>
+        <v>129.3281277734005</v>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
@@ -4265,7 +4265,7 @@
         </is>
       </c>
       <c r="B67" s="7" t="n">
-        <v>9679852.737523161</v>
+        <v>10755535.97176604</v>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
@@ -4280,7 +4280,7 @@
         </is>
       </c>
       <c r="B68" s="30" t="n">
-        <v>134.4186035896276</v>
+        <v>129.3281277734005</v>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
@@ -4310,7 +4310,7 @@
         </is>
       </c>
       <c r="B70" s="7" t="n">
-        <v>967985.2737523161</v>
+        <v>1075553.597176604</v>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
@@ -4325,7 +4325,7 @@
         </is>
       </c>
       <c r="B71" s="7" t="n">
-        <v>1943.745529623125</v>
+        <v>2159.746179069485</v>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
@@ -4340,7 +4340,7 @@
         </is>
       </c>
       <c r="B72" s="7" t="n">
-        <v>430528.3247174657</v>
+        <v>429095.4955450651</v>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
@@ -4355,7 +4355,7 @@
         </is>
       </c>
       <c r="B73" s="7" t="n">
-        <v>8281339.139053378</v>
+        <v>9250886.879044369</v>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
@@ -4370,7 +4370,7 @@
         </is>
       </c>
       <c r="B74" s="7" t="n">
-        <v>16629.19505834012</v>
+        <v>18576.07807037021</v>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
@@ -4400,7 +4400,7 @@
         </is>
       </c>
       <c r="B77" s="7" t="n">
-        <v>9218000.302959621</v>
+        <v>10293683.5372025</v>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
@@ -4415,7 +4415,7 @@
         </is>
       </c>
       <c r="B78" s="7" t="n">
-        <v>8281339.139053378</v>
+        <v>9250886.879044369</v>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
@@ -4430,7 +4430,7 @@
         </is>
       </c>
       <c r="B79" s="7" t="n">
-        <v>936661.1639062427</v>
+        <v>1042796.658158127</v>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
@@ -4445,7 +4445,7 @@
         </is>
       </c>
       <c r="B80" s="7" t="n">
-        <v>1880.845710655106</v>
+        <v>2093.969193088609</v>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
@@ -4475,7 +4475,7 @@
         </is>
       </c>
       <c r="B82" s="30" t="n">
-        <v>83.47581720581169</v>
+        <v>83.48043221691825</v>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="B84" s="7" t="n">
-        <v>1398513.598469783</v>
+        <v>1504649.092721668</v>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
@@ -4520,7 +4520,7 @@
         </is>
       </c>
       <c r="B85" s="7" t="n">
-        <v>1398513.598469782</v>
+        <v>1504649.092721669</v>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
@@ -4535,7 +4535,7 @@
         </is>
       </c>
       <c r="B86" s="9" t="n">
-        <v>1.629814505577087e-09</v>
+        <v>-1.164153218269348e-09</v>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
@@ -6254,7 +6254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34.14" customWidth="1" min="1" max="1"/>
@@ -6544,221 +6544,220 @@
           <t>Juice (lb/hr)</t>
         </is>
       </c>
-      <c r="B50" s="22" t="n">
+      <c r="B50" s="13" t="n">
         <v>1444925.45971979</v>
       </c>
-      <c r="C50" s="22" t="n">
+      <c r="C50" s="13" t="n">
         <v>481641.8199065967</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="14" t="inlineStr">
         <is>
-          <t>Duty (BTU/hr)</t>
-        </is>
-      </c>
-      <c r="B51" s="25" t="n">
-        <v>165414648.662544</v>
-      </c>
-      <c r="C51" s="25" t="n">
-        <v>55138216.220848</v>
+          <t>Juice cp (BTU/lb·°F)</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="n">
+        <v>0.9158376858810273</v>
+      </c>
+      <c r="C51" s="15" t="n">
+        <v>0.9158376858810273</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>Req Area (ft²)</t>
-        </is>
-      </c>
-      <c r="B52" s="22" t="n">
-        <v>10812.69185736374</v>
-      </c>
-      <c r="C52" s="22" t="n">
-        <v>3604.230619121246</v>
+          <t>Juice ΔT (°F)</t>
+        </is>
+      </c>
+      <c r="B52" s="13" t="n">
+        <v>125</v>
+      </c>
+      <c r="C52" s="13" t="n">
+        <v>125</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="14" t="inlineStr">
         <is>
-          <t>Inst Area (ft²)</t>
-        </is>
-      </c>
-      <c r="B53" s="25" t="n">
-        <v>11000</v>
-      </c>
-      <c r="C53" s="25" t="n">
-        <v>5000</v>
+          <t>Duty (BTU/hr)</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="n">
+        <v>165414648.662544</v>
+      </c>
+      <c r="C53" s="15" t="n">
+        <v>55138216.220848</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
+          <t>Req Area (ft²)</t>
+        </is>
+      </c>
+      <c r="B54" s="13" t="n">
+        <v>10812.69185736374</v>
+      </c>
+      <c r="C54" s="13" t="n">
+        <v>3604.230619121246</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>Inst Area (ft²)</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="n">
+        <v>11000</v>
+      </c>
+      <c r="C55" s="15" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
+        <is>
           <t>Steam (lb/hr)</t>
         </is>
       </c>
-      <c r="B54" s="22" t="n">
+      <c r="B56" s="13" t="n">
         <v>175002.5610829924</v>
       </c>
-      <c r="C54" s="22" t="n">
+      <c r="C56" s="13" t="n">
         <v>58334.1870276641</v>
       </c>
     </row>
-    <row r="56" ht="17" customHeight="1">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="58" ht="17" customHeight="1">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>HEATER CONDITIONS</t>
         </is>
       </c>
-      <c r="B56" s="5" t="n"/>
-      <c r="C56" s="5" t="n"/>
-      <c r="D56" s="5" t="n"/>
-      <c r="E56" s="5" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="11" t="inlineStr"/>
-      <c r="B57" s="11" t="inlineStr">
+      <c r="B58" s="5" t="n"/>
+      <c r="C58" s="5" t="n"/>
+      <c r="D58" s="5" t="n"/>
+      <c r="E58" s="5" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr"/>
+      <c r="B59" s="11" t="inlineStr">
         <is>
           <t>V1 Heaters</t>
         </is>
       </c>
-      <c r="C57" s="11" t="inlineStr">
+      <c r="C59" s="11" t="inlineStr">
         <is>
           <t>Exhaust Heaters</t>
         </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="12" t="inlineStr">
-        <is>
-          <t>Steam Type</t>
-        </is>
-      </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>V1</t>
-        </is>
-      </c>
-      <c r="C58" s="12" t="inlineStr">
-        <is>
-          <t>Exhaust</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="14" t="inlineStr">
-        <is>
-          <t>T in (°F)</t>
-        </is>
-      </c>
-      <c r="B59" s="15" t="n">
-        <v>95</v>
-      </c>
-      <c r="C59" s="15" t="n">
-        <v>95</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
         <is>
-          <t>T out (°F)</t>
-        </is>
-      </c>
-      <c r="B60" s="13" t="n">
-        <v>220</v>
-      </c>
-      <c r="C60" s="13" t="n">
-        <v>220</v>
+          <t>Steam Type</t>
+        </is>
+      </c>
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="C60" s="12" t="inlineStr">
+        <is>
+          <t>Exhaust</t>
+        </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="14" t="inlineStr">
         <is>
-          <t>LMTD (°F)</t>
+          <t>T in (°F)</t>
         </is>
       </c>
       <c r="B61" s="15" t="n">
-        <v>76.49096582267444</v>
+        <v>95</v>
       </c>
       <c r="C61" s="15" t="n">
-        <v>76.49096582267444</v>
+        <v>95</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
         <is>
-          <t>U (BTU/hr·ft²·°F)</t>
+          <t>T out (°F)</t>
         </is>
       </c>
       <c r="B62" s="13" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="C62" s="13" t="n">
-        <v>200</v>
+        <v>220</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="14" t="inlineStr">
         <is>
+          <t>LMTD (°F)</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="n">
+        <v>76.49096582267444</v>
+      </c>
+      <c r="C63" s="15" t="n">
+        <v>76.49096582267444</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t>U (BTU/hr·ft²·°F)</t>
+        </is>
+      </c>
+      <c r="B64" s="13" t="n">
+        <v>200</v>
+      </c>
+      <c r="C64" s="13" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
+        <is>
           <t>Steam (psia)</t>
         </is>
       </c>
-      <c r="B63" s="15" t="n">
+      <c r="B65" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="C63" s="15" t="n">
+      <c r="C65" s="15" t="n">
         <v>30</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>Total duty</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="n">
-        <v>220552864.883392</v>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>BTU/hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="6" t="inlineStr">
-        <is>
-          <t>Total steam</t>
-        </is>
-      </c>
-      <c r="B65" s="7" t="n">
-        <v>233336.7481106565</v>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>lb/hr</t>
-        </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>Juice split between heaters</t>
-        </is>
-      </c>
-      <c r="B66" s="6" t="inlineStr">
-        <is>
-          <t>75% / 25%</t>
+          <t>Total duty</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="n">
+        <v>220552864.883392</v>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>BTU/hr</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>Hot juice out</t>
+          <t>Total steam</t>
         </is>
       </c>
       <c r="B67" s="7" t="n">
-        <v>1926567.279626387</v>
+        <v>233336.7481106565</v>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
@@ -6769,69 +6768,96 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
+          <t>Juice split between heaters</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>75% / 25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>Hot juice out</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="n">
+        <v>1926567.279626387</v>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
           <t>Hot juice temperature</t>
         </is>
       </c>
-      <c r="B68" s="30" t="n">
+      <c r="B70" s="30" t="n">
         <v>220</v>
       </c>
-      <c r="C68" s="8" t="inlineStr">
+      <c r="C70" s="8" t="inlineStr">
         <is>
           <t>°F</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="17" customHeight="1">
-      <c r="A70" s="4" t="inlineStr">
+    <row r="72" ht="17" customHeight="1">
+      <c r="A72" s="4" t="inlineStr">
         <is>
           <t>CONDENSATE RETURN</t>
         </is>
       </c>
-      <c r="B70" s="5" t="n"/>
-      <c r="C70" s="5" t="n"/>
-      <c r="D70" s="5" t="n"/>
-      <c r="E70" s="5" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="6" t="inlineStr">
-        <is>
-          <t>Clean condensate (Exhaust steam heaters)</t>
-        </is>
-      </c>
-      <c r="B71" s="7" t="n">
-        <v>56030.81829974123</v>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>lb/hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="6" t="inlineStr">
-        <is>
-          <t>Dirty condensate (V1-V4 steam heaters)</t>
-        </is>
-      </c>
-      <c r="B72" s="7" t="n">
-        <v>168092.4548992238</v>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>lb/hr</t>
-        </is>
-      </c>
+      <c r="B72" s="5" t="n"/>
+      <c r="C72" s="5" t="n"/>
+      <c r="D72" s="5" t="n"/>
+      <c r="E72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
+          <t>Clean condensate (Exhaust steam heaters)</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="n">
+        <v>56030.81829974123</v>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>Dirty condensate (V1-V4 steam heaters)</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="n">
+        <v>168092.4548992238</v>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
           <t>Total condensate</t>
         </is>
       </c>
-      <c r="B73" s="7" t="n">
+      <c r="B75" s="7" t="n">
         <v>224123.273198965</v>
       </c>
-      <c r="C73" s="8" t="inlineStr">
+      <c r="C75" s="8" t="inlineStr">
         <is>
           <t>lb/hr</t>
         </is>
@@ -6842,10 +6868,10 @@
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A48:E48"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A72:E72"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A70:E70"/>
-    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A58:E58"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
@@ -6862,7 +6888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34.14" customWidth="1" min="1" max="1"/>
@@ -7041,242 +7067,262 @@
           <t>Juice (lb/hr)</t>
         </is>
       </c>
-      <c r="B44" s="22" t="n">
+      <c r="B44" s="13" t="n">
         <v>1595348.671359166</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>Duty (BTU/hr)</t>
-        </is>
-      </c>
-      <c r="B45" s="25" t="n">
-        <v>29209301.82972704</v>
+          <t>Juice cp (BTU/lb·°F)</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="n">
+        <v>0.9154519746721577</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t>Req Area (ft²)</t>
-        </is>
-      </c>
-      <c r="B46" s="22" t="n">
-        <v>4598.350953494461</v>
+          <t>Juice ΔT (°F)</t>
+        </is>
+      </c>
+      <c r="B46" s="13" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>Inst Area (ft²)</t>
-        </is>
-      </c>
-      <c r="B47" s="25" t="n">
-        <v>6000</v>
+          <t>Duty (BTU/hr)</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="n">
+        <v>29209301.82972704</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
         <is>
+          <t>Req Area (ft²)</t>
+        </is>
+      </c>
+      <c r="B48" s="13" t="n">
+        <v>4598.350953494461</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>Inst Area (ft²)</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
           <t>Steam (lb/hr)</t>
         </is>
       </c>
-      <c r="B48" s="22" t="n">
+      <c r="B50" s="13" t="n">
         <v>30902.3576145094</v>
       </c>
     </row>
-    <row r="50" ht="17" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
+    <row r="52" ht="17" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>HEATER CONDITIONS</t>
         </is>
       </c>
-      <c r="B50" s="5" t="n"/>
-      <c r="C50" s="5" t="n"/>
-      <c r="D50" s="5" t="n"/>
-      <c r="E50" s="5" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="11" t="inlineStr"/>
-      <c r="B51" s="11" t="inlineStr">
+      <c r="B52" s="5" t="n"/>
+      <c r="C52" s="5" t="n"/>
+      <c r="D52" s="5" t="n"/>
+      <c r="E52" s="5" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="inlineStr"/>
+      <c r="B53" s="11" t="inlineStr">
         <is>
           <t>Clarified Juice Heater</t>
         </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="12" t="inlineStr">
-        <is>
-          <t>Steam Type</t>
-        </is>
-      </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>Exhaust</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="14" t="inlineStr">
-        <is>
-          <t>T in (°F)</t>
-        </is>
-      </c>
-      <c r="B53" s="15" t="n">
-        <v>205</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>T out (°F)</t>
-        </is>
-      </c>
-      <c r="B54" s="13" t="n">
-        <v>225</v>
+          <t>Steam Type</t>
+        </is>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>Exhaust</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
-          <t>LMTD (°F)</t>
+          <t>T in (°F)</t>
         </is>
       </c>
       <c r="B55" s="15" t="n">
-        <v>34.33581290234913</v>
+        <v>205</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
         <is>
-          <t>U (BTU/hr·ft²·°F)</t>
+          <t>T out (°F)</t>
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>185</v>
+        <v>225</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="14" t="inlineStr">
         <is>
+          <t>LMTD (°F)</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="n">
+        <v>34.33581290234913</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
+          <t>U (BTU/hr·ft²·°F)</t>
+        </is>
+      </c>
+      <c r="B58" s="13" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="14" t="inlineStr">
+        <is>
           <t>Steam (psia)</t>
         </is>
       </c>
-      <c r="B57" s="15" t="n">
+      <c r="B59" s="15" t="n">
         <v>30</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="6" t="inlineStr">
-        <is>
-          <t>Total duty</t>
-        </is>
-      </c>
-      <c r="B58" s="7" t="n">
-        <v>29209301.82972704</v>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>BTU/hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="6" t="inlineStr">
-        <is>
-          <t>Total steam</t>
-        </is>
-      </c>
-      <c r="B59" s="7" t="n">
-        <v>30902.3576145094</v>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>lb/hr</t>
-        </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>Hot juice out</t>
+          <t>Total duty</t>
         </is>
       </c>
       <c r="B60" s="7" t="n">
-        <v>1595348.671359166</v>
+        <v>29209301.82972704</v>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>lb/hr</t>
+          <t>BTU/hr</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
+          <t>Total steam</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="n">
+        <v>30902.3576145094</v>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>Hot juice out</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="n">
+        <v>1595348.671359166</v>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
           <t>Hot juice temperature</t>
         </is>
       </c>
-      <c r="B61" s="30" t="n">
+      <c r="B63" s="30" t="n">
         <v>225</v>
       </c>
-      <c r="C61" s="8" t="inlineStr">
+      <c r="C63" s="8" t="inlineStr">
         <is>
           <t>°F</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="17" customHeight="1">
-      <c r="A63" s="4" t="inlineStr">
+    <row r="65" ht="17" customHeight="1">
+      <c r="A65" s="4" t="inlineStr">
         <is>
           <t>CONDENSATE RETURN</t>
         </is>
       </c>
-      <c r="B63" s="5" t="n"/>
-      <c r="C63" s="5" t="n"/>
-      <c r="D63" s="5" t="n"/>
-      <c r="E63" s="5" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>Clean condensate (Exhaust steam heaters)</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="n">
-        <v>29682.1550579092</v>
-      </c>
-      <c r="C64" s="8" t="inlineStr">
-        <is>
-          <t>lb/hr</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="6" t="inlineStr">
-        <is>
-          <t>Dirty condensate (V1-V4 steam heaters)</t>
-        </is>
-      </c>
-      <c r="B65" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>lb/hr</t>
-        </is>
-      </c>
+      <c r="B65" s="5" t="n"/>
+      <c r="C65" s="5" t="n"/>
+      <c r="D65" s="5" t="n"/>
+      <c r="E65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>Total condensate</t>
+          <t>Clean condensate (Exhaust steam heaters)</t>
         </is>
       </c>
       <c r="B66" s="7" t="n">
         <v>29682.1550579092</v>
       </c>
       <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>Dirty condensate (V1-V4 steam heaters)</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>lb/hr</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>Total condensate</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="n">
+        <v>29682.1550579092</v>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
         <is>
           <t>lb/hr</t>
         </is>
@@ -7285,10 +7331,10 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A65:E65"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A52:E52"/>
     <mergeCell ref="A42:E42"/>
-    <mergeCell ref="A63:E63"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:E5"/>
   </mergeCells>
@@ -12364,19 +12410,19 @@
         <v>1011.249247318053</v>
       </c>
       <c r="E267" s="33" t="n">
-        <v>86.42507599061878</v>
+        <v>86.85239436054502</v>
       </c>
       <c r="F267" s="22" t="n">
-        <v>1619785.088449194</v>
+        <v>1796107.842609179</v>
       </c>
       <c r="G267" s="22" t="n">
-        <v>3236.980592424448</v>
+        <v>3589.344209850479</v>
       </c>
       <c r="H267" s="24" t="n">
-        <v>143.355890609762</v>
+        <v>138.355890609762</v>
       </c>
       <c r="I267" s="22" t="n">
-        <v>1705248.762434443</v>
+        <v>1881571.516594429</v>
       </c>
     </row>
     <row r="268">
@@ -12395,19 +12441,19 @@
         <v>1011.249247318053</v>
       </c>
       <c r="E268" s="34" t="n">
-        <v>49.42522625424751</v>
+        <v>49.66960332738417</v>
       </c>
       <c r="F268" s="25" t="n">
-        <v>926331.2014738389</v>
+        <v>1027167.583950093</v>
       </c>
       <c r="G268" s="25" t="n">
-        <v>1851.181457781453</v>
+        <v>2052.693013489394</v>
       </c>
       <c r="H268" s="27" t="n">
-        <v>143.355890609762</v>
+        <v>138.355890609762</v>
       </c>
       <c r="I268" s="25" t="n">
-        <v>975206.6161011711</v>
+        <v>1076042.998577425</v>
       </c>
     </row>
     <row r="269">
@@ -12426,19 +12472,19 @@
         <v>1017.228576695272</v>
       </c>
       <c r="E269" s="33" t="n">
-        <v>40.07602197251683</v>
+        <v>40.27300828852613</v>
       </c>
       <c r="F269" s="22" t="n">
-        <v>930207.7255633922</v>
+        <v>1057509.698089116</v>
       </c>
       <c r="G269" s="22" t="n">
-        <v>1858.92830848</v>
+        <v>2113.328733191679</v>
       </c>
       <c r="H269" s="24" t="n">
-        <v>133.0828737186033</v>
+        <v>128.0828737186033</v>
       </c>
       <c r="I269" s="22" t="n">
-        <v>969604.9887652519</v>
+        <v>1096906.961290976</v>
       </c>
     </row>
     <row r="270">
@@ -12457,19 +12503,19 @@
         <v>1019.563890979194</v>
       </c>
       <c r="E270" s="34" t="n">
-        <v>7.962371261173675</v>
+        <v>8.001419188094305</v>
       </c>
       <c r="F270" s="25" t="n">
-        <v>203852.4787998703</v>
+        <v>234924.8969897964</v>
       </c>
       <c r="G270" s="25" t="n">
-        <v>407.3790543562556</v>
+        <v>469.4742146079064</v>
       </c>
       <c r="H270" s="27" t="n">
-        <v>129.059477265374</v>
+        <v>124.059477265374</v>
       </c>
       <c r="I270" s="25" t="n">
-        <v>211662.0641839962</v>
+        <v>242734.4823739223</v>
       </c>
     </row>
     <row r="271">
@@ -12488,19 +12534,19 @@
         <v>1024.996584701115</v>
       </c>
       <c r="E271" s="33" t="n">
-        <v>24.87623682952647</v>
+        <v>24.99758473058694</v>
       </c>
       <c r="F271" s="22" t="n">
-        <v>838057.6491100461</v>
+        <v>1012736.593040395</v>
       </c>
       <c r="G271" s="22" t="n">
-        <v>1674.775477837822</v>
+        <v>2023.854102798551</v>
       </c>
       <c r="H271" s="24" t="n">
-        <v>119.6832047961655</v>
+        <v>114.6832047961655</v>
       </c>
       <c r="I271" s="22" t="n">
-        <v>862327.2293221405</v>
+        <v>1037006.173252489</v>
       </c>
     </row>
     <row r="272">
@@ -12515,17 +12561,17 @@
       <c r="C272" s="16" t="inlineStr"/>
       <c r="D272" s="16" t="inlineStr"/>
       <c r="E272" s="35" t="n">
-        <v>208.7649323080833</v>
+        <v>209.7940098951366</v>
       </c>
       <c r="F272" s="28" t="n">
-        <v>4518234.143396341</v>
+        <v>5128446.614678579</v>
       </c>
       <c r="G272" s="28" t="n">
-        <v>9029.24489087998</v>
+        <v>10248.69427393801</v>
       </c>
       <c r="H272" s="16" t="inlineStr"/>
       <c r="I272" s="28" t="n">
-        <v>4724049.660807002</v>
+        <v>5334262.132089241</v>
       </c>
     </row>
     <row r="273">
@@ -12979,7 +13025,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>3 sets  |  total steam = 288,279 lb/hr  |  total condenser injection water = 6,084,253 lb/hr (12,159 GPM)</t>
+          <t>3 sets  |  total steam = 288,279 lb/hr  |  total condenser injection water = 6,922,616 lb/hr (13,834 GPM)</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -13812,7 +13858,7 @@
         </is>
       </c>
       <c r="B81" s="7" t="n">
-        <v>143472412.6263661</v>
+        <v>144177516.4375404</v>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
@@ -13842,7 +13888,7 @@
         </is>
       </c>
       <c r="B83" s="30" t="n">
-        <v>132.8134936467732</v>
+        <v>127.8134936467732</v>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
@@ -13857,7 +13903,7 @@
         </is>
       </c>
       <c r="B84" s="7" t="n">
-        <v>3351102.664269011</v>
+        <v>3812858.917093043</v>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
@@ -13872,7 +13918,7 @@
         </is>
       </c>
       <c r="B85" s="7" t="n">
-        <v>6696.847850257815</v>
+        <v>7619.622136476904</v>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
@@ -13887,7 +13933,7 @@
         </is>
       </c>
       <c r="B86" s="7" t="n">
-        <v>3492123.426503871</v>
+        <v>3953879.679327903</v>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
@@ -14783,7 +14829,7 @@
         </is>
       </c>
       <c r="B171" s="7" t="n">
-        <v>68128571.9476818</v>
+        <v>68463393.9169427</v>
       </c>
       <c r="C171" s="8" t="inlineStr">
         <is>
@@ -14813,7 +14859,7 @@
         </is>
       </c>
       <c r="B173" s="30" t="n">
-        <v>132.8134936467732</v>
+        <v>127.8134936467732</v>
       </c>
       <c r="C173" s="8" t="inlineStr">
         <is>
@@ -14828,7 +14874,7 @@
         </is>
       </c>
       <c r="B174" s="7" t="n">
-        <v>1591287.375652338</v>
+        <v>1810554.574948273</v>
       </c>
       <c r="C174" s="8" t="inlineStr">
         <is>
@@ -14843,7 +14889,7 @@
         </is>
       </c>
       <c r="B175" s="7" t="n">
-        <v>3180.030726723297</v>
+        <v>3618.214578233958</v>
       </c>
       <c r="C175" s="8" t="inlineStr">
         <is>
@@ -14858,7 +14904,7 @@
         </is>
       </c>
       <c r="B176" s="7" t="n">
-        <v>1658251.769504519</v>
+        <v>1877518.968800454</v>
       </c>
       <c r="C176" s="8" t="inlineStr">
         <is>
@@ -15656,7 +15702,7 @@
         </is>
       </c>
       <c r="B266" s="7" t="n">
-        <v>48887142.44488114</v>
+        <v>49127401.25021033</v>
       </c>
       <c r="C266" s="8" t="inlineStr">
         <is>
@@ -15686,7 +15732,7 @@
         </is>
       </c>
       <c r="B268" s="30" t="n">
-        <v>132.8134936467732</v>
+        <v>127.8134936467732</v>
       </c>
       <c r="C268" s="8" t="inlineStr">
         <is>
@@ -15701,7 +15747,7 @@
         </is>
       </c>
       <c r="B269" s="7" t="n">
-        <v>1141862.956763533</v>
+        <v>1299202.917062456</v>
       </c>
       <c r="C269" s="8" t="inlineStr">
         <is>
@@ -15716,7 +15762,7 @@
         </is>
       </c>
       <c r="B270" s="7" t="n">
-        <v>2281.900393212496</v>
+        <v>2596.328771108025</v>
       </c>
       <c r="C270" s="8" t="inlineStr">
         <is>
@@ -15731,7 +15777,7 @@
         </is>
       </c>
       <c r="B271" s="7" t="n">
-        <v>1189914.71782937</v>
+        <v>1347254.678128293</v>
       </c>
       <c r="C271" s="8" t="inlineStr">
         <is>

</xml_diff>